<commit_message>
Added Advanced level of SQL injection
</commit_message>
<xml_diff>
--- a/Testing Documentation.xlsx
+++ b/Testing Documentation.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MAMP\htdocs\Education-System\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{857DC0AE-0483-4760-ADAE-1B2C5B051487}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C3DD100-1087-4F24-8577-E63F141EF5DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="126">
   <si>
     <t>Test ID</t>
   </si>
@@ -313,13 +313,103 @@
   </si>
   <si>
     <t>Test was performed according to your update. Confirm the response"Invalid input" and that no comment was added.</t>
+  </si>
+  <si>
+    <t>SQL-01</t>
+  </si>
+  <si>
+    <t>SQL-Injection Easy level</t>
+  </si>
+  <si>
+    <t>SQL-02</t>
+  </si>
+  <si>
+    <t>evidence/vulnerable/vulnerable-easy-sql-injection.png</t>
+  </si>
+  <si>
+    <t>evidence/safe/safe-easy-sql-injection.png</t>
+  </si>
+  <si>
+    <t>Confirms normal functionality in Safe mode.</t>
+  </si>
+  <si>
+    <t>SQL-03</t>
+  </si>
+  <si>
+    <t>SQL-Injection Intermediate level</t>
+  </si>
+  <si>
+    <t>evidence/vulnerable/vulnerable-intermediate-sql-injection.png</t>
+  </si>
+  <si>
+    <t>SQL-04</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> OR '1'='1'</t>
+  </si>
+  <si>
+    <t>1 OR 1=1</t>
+  </si>
+  <si>
+    <t>Show all the comments</t>
+  </si>
+  <si>
+    <t>Tests showed that all comments are visible</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Show no matching found </t>
+  </si>
+  <si>
+    <t>Tests showed that no comments are visible with no matching found text</t>
+  </si>
+  <si>
+    <t>Show no matching comments found</t>
+  </si>
+  <si>
+    <t>evidence/safe/safe-intermediate-sql-injection.png</t>
+  </si>
+  <si>
+    <t>Normal ID lookup.</t>
+  </si>
+  <si>
+    <t>SQL-05</t>
+  </si>
+  <si>
+    <t>SQL-06</t>
+  </si>
+  <si>
+    <t>SQL-Injection Advance Level</t>
+  </si>
+  <si>
+    <t>evidence/vulnerable/vunerable-sqli-advanced-safe-mode.png</t>
+  </si>
+  <si>
+    <t>evidence/safe/safe-sqli-advanced-safe-mode.png</t>
+  </si>
+  <si>
+    <t>The advanced lab’s prepared statement alone does not prove all application routes are safe.</t>
+  </si>
+  <si>
+    <t>Direct lab query; not proof of a successful injection chain.</t>
+  </si>
+  <si>
+    <t>Fail</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> UNION SELECT 999, 'LAB_MARKER', '2000-01-01', 'Lab User', 'Synthetic Result' #</t>
+  </si>
+  <si>
+    <t>' UNION SELECT 999, 'LAB_MARKER', '2000-01-01', 'Lab User', 'Synthetic Result' #</t>
+  </si>
+  <si>
+    <t>Show all comments</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -366,6 +456,27 @@
     </font>
     <font>
       <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF174A5B"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -438,7 +549,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -458,11 +569,6 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -470,11 +576,33 @@
     <xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -777,68 +905,69 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="2" width="23" customWidth="1"/>
+    <col min="2" max="2" width="31.7265625" customWidth="1"/>
     <col min="3" max="3" width="16" customWidth="1"/>
-    <col min="4" max="6" width="43" customWidth="1"/>
+    <col min="4" max="5" width="43" customWidth="1"/>
+    <col min="6" max="6" width="65.36328125" customWidth="1"/>
     <col min="7" max="7" width="23" customWidth="1"/>
-    <col min="8" max="8" width="34" customWidth="1"/>
+    <col min="8" max="8" width="49.36328125" customWidth="1"/>
     <col min="9" max="9" width="42" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="15"/>
-      <c r="G1" s="15"/>
-      <c r="H1" s="15"/>
-      <c r="I1" s="15"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
+      <c r="I1" s="12"/>
     </row>
     <row r="2" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="8"/>
-      <c r="B2" s="7"/>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
-      <c r="H2" s="7"/>
-      <c r="I2" s="7"/>
-    </row>
-    <row r="3" spans="1:9" s="13" customFormat="1" ht="32" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="12" t="s">
+      <c r="A2" s="13"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+      <c r="H2" s="14"/>
+      <c r="I2" s="14"/>
+    </row>
+    <row r="3" spans="1:9" s="10" customFormat="1" ht="32" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="12" t="s">
+      <c r="C3" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="12" t="s">
+      <c r="D3" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="12" t="s">
+      <c r="E3" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="F3" s="12" t="s">
+      <c r="F3" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="G3" s="12" t="s">
+      <c r="G3" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="H3" s="12" t="s">
+      <c r="H3" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="I3" s="12" t="s">
+      <c r="I3" s="9" t="s">
         <v>8</v>
       </c>
     </row>
@@ -861,7 +990,7 @@
       <c r="F4" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="G4" s="10" t="s">
+      <c r="G4" s="7" t="s">
         <v>15</v>
       </c>
       <c r="H4" s="3" t="s">
@@ -890,7 +1019,7 @@
       <c r="F5" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="G5" s="10" t="s">
+      <c r="G5" s="7" t="s">
         <v>15</v>
       </c>
       <c r="H5" s="3" t="s">
@@ -919,7 +1048,7 @@
       <c r="F6" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="G6" s="10" t="s">
+      <c r="G6" s="7" t="s">
         <v>15</v>
       </c>
       <c r="H6" s="3" t="s">
@@ -948,7 +1077,7 @@
       <c r="F7" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="G7" s="10" t="s">
+      <c r="G7" s="7" t="s">
         <v>15</v>
       </c>
       <c r="H7" s="3" t="s">
@@ -977,7 +1106,7 @@
       <c r="F8" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="G8" s="10" t="s">
+      <c r="G8" s="7" t="s">
         <v>15</v>
       </c>
       <c r="H8" s="3" t="s">
@@ -1006,7 +1135,7 @@
       <c r="F9" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="G9" s="10" t="s">
+      <c r="G9" s="7" t="s">
         <v>15</v>
       </c>
       <c r="H9" s="3" t="s">
@@ -1035,7 +1164,7 @@
       <c r="F10" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="G10" s="10" t="s">
+      <c r="G10" s="7" t="s">
         <v>15</v>
       </c>
       <c r="H10" s="3" t="s">
@@ -1046,7 +1175,7 @@
       </c>
     </row>
     <row r="11" spans="1:9" ht="88" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="21" t="s">
         <v>49</v>
       </c>
       <c r="B11" s="3" t="s">
@@ -1064,7 +1193,7 @@
       <c r="F11" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="G11" s="10" t="s">
+      <c r="G11" s="7" t="s">
         <v>15</v>
       </c>
       <c r="H11" s="3" t="s">
@@ -1074,8 +1203,173 @@
         <v>52</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="G12" s="11"/>
+    <row r="12" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="A12" s="16" t="s">
+        <v>96</v>
+      </c>
+      <c r="B12" s="17" t="s">
+        <v>97</v>
+      </c>
+      <c r="C12" s="18" t="s">
+        <v>11</v>
+      </c>
+      <c r="D12" s="22" t="s">
+        <v>106</v>
+      </c>
+      <c r="E12" t="s">
+        <v>108</v>
+      </c>
+      <c r="F12" t="s">
+        <v>109</v>
+      </c>
+      <c r="G12" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="H12" s="17" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="35" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="16" t="s">
+        <v>98</v>
+      </c>
+      <c r="B13" t="s">
+        <v>97</v>
+      </c>
+      <c r="C13" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="D13" s="22" t="s">
+        <v>106</v>
+      </c>
+      <c r="E13" t="s">
+        <v>110</v>
+      </c>
+      <c r="F13" t="s">
+        <v>111</v>
+      </c>
+      <c r="G13" s="20" t="s">
+        <v>15</v>
+      </c>
+      <c r="H13" t="s">
+        <v>100</v>
+      </c>
+      <c r="I13" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="A14" s="16" t="s">
+        <v>102</v>
+      </c>
+      <c r="B14" t="s">
+        <v>103</v>
+      </c>
+      <c r="C14" s="18" t="s">
+        <v>11</v>
+      </c>
+      <c r="D14" t="s">
+        <v>107</v>
+      </c>
+      <c r="E14" t="s">
+        <v>108</v>
+      </c>
+      <c r="F14" t="s">
+        <v>109</v>
+      </c>
+      <c r="G14" s="20" t="s">
+        <v>15</v>
+      </c>
+      <c r="H14" s="17" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="39" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="16" t="s">
+        <v>105</v>
+      </c>
+      <c r="B15" t="s">
+        <v>103</v>
+      </c>
+      <c r="C15" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="D15" t="s">
+        <v>107</v>
+      </c>
+      <c r="E15" t="s">
+        <v>112</v>
+      </c>
+      <c r="F15" t="s">
+        <v>111</v>
+      </c>
+      <c r="G15" s="20" t="s">
+        <v>15</v>
+      </c>
+      <c r="H15" t="s">
+        <v>113</v>
+      </c>
+      <c r="I15" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="34" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="16" t="s">
+        <v>115</v>
+      </c>
+      <c r="B16" t="s">
+        <v>117</v>
+      </c>
+      <c r="C16" s="18" t="s">
+        <v>11</v>
+      </c>
+      <c r="D16" s="22" t="s">
+        <v>123</v>
+      </c>
+      <c r="E16" s="22" t="s">
+        <v>125</v>
+      </c>
+      <c r="F16" t="s">
+        <v>111</v>
+      </c>
+      <c r="G16" s="20" t="s">
+        <v>122</v>
+      </c>
+      <c r="H16" t="s">
+        <v>118</v>
+      </c>
+      <c r="I16" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" ht="23" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="16" t="s">
+        <v>116</v>
+      </c>
+      <c r="B17" t="s">
+        <v>117</v>
+      </c>
+      <c r="C17" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="D17" t="s">
+        <v>124</v>
+      </c>
+      <c r="E17" t="s">
+        <v>112</v>
+      </c>
+      <c r="F17" t="s">
+        <v>111</v>
+      </c>
+      <c r="G17" s="20" t="s">
+        <v>15</v>
+      </c>
+      <c r="H17" t="s">
+        <v>119</v>
+      </c>
+      <c r="I17" t="s">
+        <v>120</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A3:I11" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
@@ -1083,6 +1377,7 @@
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:I2"/>
   </mergeCells>
+  <phoneticPr fontId="10" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1099,12 +1394,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
@@ -1236,10 +1531,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="21" x14ac:dyDescent="0.5">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="15" t="s">
         <v>68</v>
       </c>
-      <c r="B1" s="7"/>
+      <c r="B1" s="14"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="s">

</xml_diff>